<commit_message>
Migrate visualization notebooks and clean repo
Move visualization- and reasoning-focused notebooks out of the main analysis repo (several notebooks deleted/archived and extract_nnt_lrs.ipynb renamed into archive/). Remove the generated report example (reports/display_reasoning.html) and add reports/.gitkeep placeholder. Update README to reflect reduced dependency surface (remove pystata note, add test_notebook_dependencies reference) and document the migration in docs/DECISIONS.md. Also add notebooks/new-dataset.jsonl and update processed data (completed_lrs.xlsx). This tidies the repository scope and lowers notebook-related dependencies.
</commit_message>
<xml_diff>
--- a/data/processed/assessments/completed_lrs.xlsx
+++ b/data/processed/assessments/completed_lrs.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cardiac" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GERD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esophageal Dysphagia" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CREST" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cardiac" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GERD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Esophageal Dysphagia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CREST" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,16 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,12 +421,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
@@ -626,7 +614,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>WEAK NEGATIVE</t>
         </is>
       </c>
     </row>
@@ -689,12 +677,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
@@ -780,7 +768,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>STRONG POSITIVE</t>
+          <t>WEAK POSITIVE</t>
         </is>
       </c>
     </row>
@@ -792,7 +780,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>WEAK NEGATIVE</t>
         </is>
       </c>
     </row>
@@ -847,12 +835,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
@@ -878,7 +866,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>STRONG POSITIVE</t>
+          <t>WEAK POSITIVE</t>
         </is>
       </c>
     </row>
@@ -902,7 +890,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>WEAK NEGATIVE</t>
+          <t>WEAK POSITIVE</t>
         </is>
       </c>
     </row>
@@ -950,7 +938,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>WEAK NEGATIVE</t>
         </is>
       </c>
     </row>
@@ -981,12 +969,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
@@ -1081,12 +1069,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Information</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
@@ -1180,7 +1168,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WEAK POSITIVE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1180,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WEAK NEGATIVE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
     </row>

</xml_diff>